<commit_message>
A2 - Problema 1
</commit_message>
<xml_diff>
--- a/2024_1_SPCE_Avaliacao_A2_-_Felipe_Luiza_Marcius.xlsx
+++ b/2024_1_SPCE_Avaliacao_A2_-_Felipe_Luiza_Marcius.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\EngenhariaSoftwarePUCRS\Sistemas_de_Planejamento_e_Custos_para_Engenharia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mithra\Documents\FelipeFreitas\Sistemas_de_Planejamento_e_Custos_para_Engenharia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B41632A2-3780-44E8-B84F-1F068764FA18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB88AEF3-6A00-41FD-B797-229652444E37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="16200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Integrantes" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="58">
   <si>
     <t>Integrantes</t>
   </si>
@@ -166,9 +166,6 @@
     <t>(1 peça metálicas)</t>
   </si>
   <si>
-    <t>Tempo de produção de 1 peça:</t>
-  </si>
-  <si>
     <t>Peças produzidas por hora</t>
   </si>
   <si>
@@ -200,6 +197,21 @@
   </si>
   <si>
     <t>kWh. Total =</t>
+  </si>
+  <si>
+    <t>Custo total unitário de produção de 4000 peças por mês:</t>
+  </si>
+  <si>
+    <t>Custo direto unitário:</t>
+  </si>
+  <si>
+    <t>Custo direto unitário de produção de 6000 peças por mês:</t>
+  </si>
+  <si>
+    <t>Custo Direto Total</t>
+  </si>
+  <si>
+    <t>Custo Direto Unitário</t>
   </si>
 </sst>
 </file>
@@ -376,7 +388,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -438,9 +450,17 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Currency" xfId="1" builtinId="4"/>
+    <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1211,7 +1231,7 @@
         <v>90</v>
       </c>
       <c r="E9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.25">
@@ -1394,7 +1414,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8092ED7-22EC-44F0-9820-AE611F649C3D}">
-  <dimension ref="B2:H32"/>
+  <dimension ref="B2:J37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.7109375" customWidth="1"/>
@@ -1403,6 +1423,8 @@
     <col min="5" max="5" width="28.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
@@ -1455,7 +1477,7 @@
         <v>0</v>
       </c>
       <c r="F5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G5">
         <f>C5+D5+E5</f>
@@ -1479,7 +1501,7 @@
         <v>6.6666666666666666E-2</v>
       </c>
       <c r="F6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G6" s="20">
         <f>C6+D6+E6</f>
@@ -1503,7 +1525,7 @@
         <v>10</v>
       </c>
       <c r="F7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G7" s="12">
         <f>C7+D7+E7</f>
@@ -1514,246 +1536,400 @@
       <c r="B10" t="s">
         <v>42</v>
       </c>
-      <c r="C10" s="20">
-        <f>C6+D6+E6</f>
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="D10" t="s">
-        <v>30</v>
+      <c r="C10">
+        <f>1/G6</f>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="C11">
-        <f>1/C10</f>
-        <v>3</v>
+        <f>'Problema 1 (enunciado)'!C22</f>
+        <v>800</v>
+      </c>
+      <c r="D11" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="C12">
-        <v>800</v>
-      </c>
-      <c r="D12" t="s">
-        <v>38</v>
+        <f>C10*C11</f>
+        <v>2400</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
+      <c r="C13" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="21">
+        <v>4</v>
+      </c>
+      <c r="D14" s="21">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="12">
+        <v>272000</v>
+      </c>
+      <c r="D16" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C17">
+        <v>76000</v>
+      </c>
+      <c r="D17" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B19" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+    </row>
+    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B21" s="4"/>
+      <c r="C21" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C13">
-        <f>C11*C12</f>
-        <v>2400</v>
-      </c>
-    </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C14" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="D14" s="21" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B15" t="s">
-        <v>22</v>
-      </c>
-      <c r="C15" s="21">
-        <v>4</v>
-      </c>
-      <c r="D15" s="21">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B17" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17" s="12">
-        <v>272000</v>
-      </c>
-      <c r="D17" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="C18">
-        <v>76000</v>
-      </c>
-      <c r="D18" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B20" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="H20" s="5" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-    </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B22" s="4"/>
-      <c r="C22" s="5" t="s">
+      <c r="E21" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="F21" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+    </row>
+    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B23" s="2"/>
+      <c r="C23" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="E22" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F22" s="5" t="s">
+      <c r="E23" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="G22" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="H22" s="5" t="s">
+      <c r="G23" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="H23" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-    </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B24" s="2"/>
-      <c r="C24" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="E24" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="G24" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="H24" s="9" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B26" s="23" t="s">
+    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B25" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C26" s="9" t="str">
+      <c r="C25" s="9" t="str">
         <f>'Problema 1 (enunciado)'!C8</f>
         <v>-</v>
       </c>
-      <c r="D26" s="24">
+      <c r="D25" s="24">
         <f>'Problema 1 (enunciado)'!D8*'Problema 1'!G5</f>
         <v>80</v>
       </c>
-      <c r="E26" s="22"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="22"/>
-      <c r="H26" s="22"/>
-    </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B27" s="23" t="s">
+      <c r="E25" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F25" s="28">
+        <f>D25</f>
+        <v>80</v>
+      </c>
+      <c r="G25" s="22"/>
+      <c r="H25" s="28">
+        <f>D25</f>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="26" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B26" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="C27" s="25">
+      <c r="C26" s="25">
         <f>'Problema 1 (enunciado)'!C9</f>
         <v>80000</v>
       </c>
-      <c r="D27" s="24">
+      <c r="D26" s="24">
         <f>'Problema 1 (enunciado)'!D9*'Problema 1'!G6</f>
         <v>30</v>
       </c>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="22"/>
-      <c r="H27" s="22"/>
-    </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B28" s="23" t="s">
+      <c r="E26" s="22">
+        <f>C26*1.2</f>
+        <v>96000</v>
+      </c>
+      <c r="F26" s="28">
+        <f t="shared" ref="F26:F29" si="0">D26</f>
+        <v>30</v>
+      </c>
+      <c r="G26" s="25">
+        <f>C26*1.5</f>
+        <v>120000</v>
+      </c>
+      <c r="H26" s="28">
+        <f t="shared" ref="H26:H29" si="1">D26</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B27" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="C28" s="25">
+      <c r="C27" s="25">
         <f>'Problema 1 (enunciado)'!C10</f>
         <v>20000</v>
       </c>
-      <c r="D28" s="24">
+      <c r="D27" s="24">
         <f>'Problema 1 (enunciado)'!D10*'Problema 1'!G7</f>
         <v>90</v>
       </c>
-      <c r="E28" s="22"/>
-      <c r="F28" s="22"/>
-      <c r="G28" s="22"/>
-      <c r="H28" s="22"/>
-    </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B29" s="23" t="s">
+      <c r="E27" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F27" s="28">
+        <f t="shared" si="0"/>
+        <v>90</v>
+      </c>
+      <c r="G27" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="H27" s="28">
+        <f t="shared" si="1"/>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="28" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B28" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="C29" s="25">
+      <c r="C28" s="25">
         <f>'Problema 1 (enunciado)'!C11</f>
         <v>32000</v>
       </c>
-      <c r="D29" s="9"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="22"/>
-      <c r="G29" s="22"/>
-      <c r="H29" s="22"/>
-    </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B30" s="23" t="s">
+      <c r="D28" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F28" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G28" s="25">
+        <v>24000</v>
+      </c>
+      <c r="H28" s="28" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="29" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B29" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="C30" s="25">
+      <c r="C29" s="25">
         <f>'Problema 1 (enunciado)'!C12</f>
         <v>60000</v>
       </c>
-      <c r="D30" s="9"/>
-      <c r="E30" s="22"/>
-      <c r="F30" s="22"/>
-      <c r="G30" s="22"/>
-      <c r="H30" s="22"/>
-    </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B32" s="4" t="s">
-        <v>49</v>
+      <c r="D29" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F29" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G29" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="H29" s="28" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="31" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B31" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C31" s="10">
+        <f>SUM(C25:C29)</f>
+        <v>192000</v>
+      </c>
+      <c r="D31" s="10">
+        <f t="shared" ref="D31:H31" si="2">SUM(D25:D29)</f>
+        <v>200</v>
+      </c>
+      <c r="E31" s="10">
+        <f t="shared" si="2"/>
+        <v>96000</v>
+      </c>
+      <c r="F31" s="10">
+        <f t="shared" si="2"/>
+        <v>200</v>
+      </c>
+      <c r="G31" s="10">
+        <f t="shared" si="2"/>
+        <v>144000</v>
+      </c>
+      <c r="H31" s="10">
+        <f t="shared" si="2"/>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="32" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="I32" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="33" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="B33" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="C33" s="30">
+        <f>C12*D31+C31</f>
+        <v>672000</v>
+      </c>
+      <c r="D33" s="30"/>
+      <c r="E33" s="30">
+        <f>(4000-C12)*F31+E31</f>
+        <v>416000</v>
+      </c>
+      <c r="G33" s="30"/>
+      <c r="I33" s="30">
+        <f>C33+E33+G33</f>
+        <v>1088000</v>
+      </c>
+      <c r="J33" s="30">
+        <f>I33/4000</f>
+        <v>272</v>
+      </c>
+    </row>
+    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
+        <v>54</v>
+      </c>
+      <c r="C34" s="30">
+        <f>C33/C12</f>
+        <v>280</v>
+      </c>
+      <c r="E34" s="30">
+        <f>E33/(4000-C12)</f>
+        <v>260</v>
+      </c>
+      <c r="G34" s="30"/>
+    </row>
+    <row r="36" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="B36" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="C36" s="30">
+        <f>C12*D31+C31</f>
+        <v>672000</v>
+      </c>
+      <c r="E36" s="30">
+        <f>C12*F31+E31</f>
+        <v>576000</v>
+      </c>
+      <c r="G36" s="30">
+        <f>(6000-C12-C12)*H31+G31</f>
+        <v>384000</v>
+      </c>
+      <c r="I36" s="30">
+        <f>C36+E36+G36</f>
+        <v>1632000</v>
+      </c>
+      <c r="J36" s="30">
+        <f>I36/6000</f>
+        <v>272</v>
+      </c>
+    </row>
+    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B37" t="s">
+        <v>54</v>
+      </c>
+      <c r="C37" s="30">
+        <f>C36/C12</f>
+        <v>280</v>
+      </c>
+      <c r="E37" s="30">
+        <f>E36/C12</f>
+        <v>240</v>
+      </c>
+      <c r="G37" s="30">
+        <f>G36/(6000-C12-C12)</f>
+        <v>320</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
A2 - Problema 1 - Revisado
A fazer: Gráficos e Análise
</commit_message>
<xml_diff>
--- a/2024_1_SPCE_Avaliacao_A2_-_Felipe_Luiza_Marcius.xlsx
+++ b/2024_1_SPCE_Avaliacao_A2_-_Felipe_Luiza_Marcius.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mithra\Documents\FelipeFreitas\Sistemas_de_Planejamento_e_Custos_para_Engenharia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB88AEF3-6A00-41FD-B797-229652444E37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A9ED4FC-6B19-4F49-AA75-99A324DBD05A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Integrantes" sheetId="1" r:id="rId1"/>
     <sheet name="Problema 1 (enunciado)" sheetId="10" r:id="rId2"/>
-    <sheet name="Problema 1" sheetId="11" r:id="rId3"/>
+    <sheet name="Problema 1 (calculos)" sheetId="11" r:id="rId3"/>
+    <sheet name="Problema 1 (graficos)" sheetId="12" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="61">
   <si>
     <t>Integrantes</t>
   </si>
@@ -212,6 +213,15 @@
   </si>
   <si>
     <t>Custo Direto Unitário</t>
+  </si>
+  <si>
+    <t>Custo fixo de armazenagem para 3º mês</t>
+  </si>
+  <si>
+    <t>Custo Total Unitário</t>
+  </si>
+  <si>
+    <t>Custo Total</t>
   </si>
 </sst>
 </file>
@@ -1156,7 +1166,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43707723-EC2D-4934-97D3-53388F7C676B}">
-  <dimension ref="B2:F27"/>
+  <dimension ref="B2:F28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="34.7109375" bestFit="1" customWidth="1"/>
@@ -1214,6 +1224,7 @@
         <v>19</v>
       </c>
       <c r="D8" s="10">
+        <f>16</f>
         <v>16</v>
       </c>
       <c r="E8" t="s">
@@ -1225,9 +1236,11 @@
         <v>15</v>
       </c>
       <c r="C9" s="11">
+        <f>80000</f>
         <v>80000</v>
       </c>
       <c r="D9" s="10">
+        <f>90</f>
         <v>90</v>
       </c>
       <c r="E9" t="s">
@@ -1239,9 +1252,11 @@
         <v>16</v>
       </c>
       <c r="C10" s="11">
+        <f>20000</f>
         <v>20000</v>
       </c>
       <c r="D10" s="10">
+        <f>4.5</f>
         <v>4.5</v>
       </c>
       <c r="E10" t="s">
@@ -1253,6 +1268,7 @@
         <v>17</v>
       </c>
       <c r="C11" s="11">
+        <f>32000</f>
         <v>32000</v>
       </c>
       <c r="D11" t="s">
@@ -1264,6 +1280,7 @@
         <v>18</v>
       </c>
       <c r="C12" s="11">
+        <f>60000</f>
         <v>60000</v>
       </c>
       <c r="D12" t="s">
@@ -1389,20 +1406,31 @@
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
+        <v>58</v>
+      </c>
+      <c r="C26">
+        <f>24000</f>
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
         <v>35</v>
       </c>
-      <c r="C26" s="12">
+      <c r="C27" s="12">
+        <f>272000</f>
         <v>272000</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D27" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C27">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C28">
+        <f>76000</f>
         <v>76000</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D28" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1414,17 +1442,19 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8092ED7-22EC-44F0-9820-AE611F649C3D}">
-  <dimension ref="B2:J37"/>
+  <dimension ref="B2:L37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.7109375" customWidth="1"/>
+    <col min="1" max="1" width="3.7109375" customWidth="1"/>
     <col min="2" max="2" width="34.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="27.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="28.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="24" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
@@ -1592,7 +1622,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="C17">
         <v>76000</v>
       </c>
@@ -1600,7 +1630,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="8" t="s">
         <v>9</v>
       </c>
@@ -1623,7 +1653,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -1632,7 +1662,7 @@
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
     </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="4"/>
       <c r="C21" s="5" t="s">
         <v>11</v>
@@ -1653,7 +1683,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
@@ -1662,7 +1692,7 @@
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
     </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="2"/>
       <c r="C23" s="9" t="s">
         <v>13</v>
@@ -1683,7 +1713,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="23" t="s">
         <v>14</v>
       </c>
@@ -1692,7 +1722,7 @@
         <v>-</v>
       </c>
       <c r="D25" s="24">
-        <f>'Problema 1 (enunciado)'!D8*'Problema 1'!G5</f>
+        <f>'Problema 1 (enunciado)'!D8*'Problema 1 (calculos)'!G5</f>
         <v>80</v>
       </c>
       <c r="E25" s="9" t="s">
@@ -1708,7 +1738,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="23" t="s">
         <v>15</v>
       </c>
@@ -1717,7 +1747,7 @@
         <v>80000</v>
       </c>
       <c r="D26" s="24">
-        <f>'Problema 1 (enunciado)'!D9*'Problema 1'!G6</f>
+        <f>'Problema 1 (enunciado)'!D9*'Problema 1 (calculos)'!G6</f>
         <v>30</v>
       </c>
       <c r="E26" s="22">
@@ -1737,7 +1767,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="23" t="s">
         <v>16</v>
       </c>
@@ -1746,7 +1776,7 @@
         <v>20000</v>
       </c>
       <c r="D27" s="24">
-        <f>'Problema 1 (enunciado)'!D10*'Problema 1'!G7</f>
+        <f>'Problema 1 (enunciado)'!D10*'Problema 1 (calculos)'!G7</f>
         <v>90</v>
       </c>
       <c r="E27" s="9" t="s">
@@ -1764,7 +1794,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="23" t="s">
         <v>17</v>
       </c>
@@ -1783,6 +1813,7 @@
         <v>-</v>
       </c>
       <c r="G28" s="25">
+        <f>'Problema 1 (enunciado)'!C26</f>
         <v>24000</v>
       </c>
       <c r="H28" s="28" t="str">
@@ -1790,7 +1821,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="23" t="s">
         <v>18</v>
       </c>
@@ -1816,7 +1847,7 @@
         <v>-</v>
       </c>
     </row>
-    <row r="31" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="4" t="s">
         <v>48</v>
       </c>
@@ -1845,15 +1876,21 @@
         <v>200</v>
       </c>
     </row>
-    <row r="32" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="I32" s="1" t="s">
         <v>56</v>
       </c>
       <c r="J32" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="33" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K32" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="L32" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="33" spans="2:12" ht="30" x14ac:dyDescent="0.25">
       <c r="B33" s="29" t="s">
         <v>53</v>
       </c>
@@ -1875,8 +1912,16 @@
         <f>I33/4000</f>
         <v>272</v>
       </c>
-    </row>
-    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="K33" s="30">
+        <f>I33+'Problema 1 (enunciado)'!C27</f>
+        <v>1360000</v>
+      </c>
+      <c r="L33" s="30">
+        <f>K33/4000</f>
+        <v>340</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>54</v>
       </c>
@@ -1890,7 +1935,7 @@
       </c>
       <c r="G34" s="30"/>
     </row>
-    <row r="36" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:12" ht="30" x14ac:dyDescent="0.25">
       <c r="B36" s="29" t="s">
         <v>55</v>
       </c>
@@ -1914,8 +1959,16 @@
         <f>I36/6000</f>
         <v>272</v>
       </c>
-    </row>
-    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="K36" s="30">
+        <f>I36+'Problema 1 (enunciado)'!C27+'Problema 1 (enunciado)'!C28</f>
+        <v>1980000</v>
+      </c>
+      <c r="L36" s="30">
+        <f>K36/6000</f>
+        <v>330</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>54</v>
       </c>
@@ -1935,5 +1988,562 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="K33 K36" formula="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460B9E08-268A-41C8-B869-A106BBCA7C13}">
+  <dimension ref="B2:L37"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="3.7109375" customWidth="1"/>
+    <col min="2" max="2" width="34.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="24" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B2" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" ht="3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="15"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="16"/>
+    </row>
+    <row r="4" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5">
+        <f>'Problema 1 (enunciado)'!C18/9</f>
+        <v>3</v>
+      </c>
+      <c r="D5">
+        <f>'Problema 1 (enunciado)'!D18/6</f>
+        <v>2</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" t="s">
+        <v>50</v>
+      </c>
+      <c r="G5">
+        <f>C5+D5+E5</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="20">
+        <f>'Problema 1 (enunciado)'!C19/9</f>
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D6">
+        <f>'Problema 1 (enunciado)'!D19/6</f>
+        <v>9.9999999999999992E-2</v>
+      </c>
+      <c r="E6" s="20">
+        <f>'Problema 1 (enunciado)'!E19/12</f>
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="F6" t="s">
+        <v>51</v>
+      </c>
+      <c r="G6" s="20">
+        <f>C6+D6+E6</f>
+        <v>0.33333333333333331</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="12">
+        <f>'Problema 1 (enunciado)'!C20/9</f>
+        <v>5</v>
+      </c>
+      <c r="D7" s="12">
+        <f>'Problema 1 (enunciado)'!D20/6</f>
+        <v>5</v>
+      </c>
+      <c r="E7" s="12">
+        <f>'Problema 1 (enunciado)'!E20/12</f>
+        <v>10</v>
+      </c>
+      <c r="F7" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" s="12">
+        <f>C7+D7+E7</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10">
+        <f>1/G6</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11">
+        <f>'Problema 1 (enunciado)'!C22</f>
+        <v>800</v>
+      </c>
+      <c r="D11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12">
+        <f>C10*C11</f>
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C13" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="21">
+        <v>4</v>
+      </c>
+      <c r="D14" s="21">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="12">
+        <v>272000</v>
+      </c>
+      <c r="D16" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="C17">
+        <v>76000</v>
+      </c>
+      <c r="D17" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B19" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B21" s="4"/>
+      <c r="C21" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B23" s="2"/>
+      <c r="C23" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="G23" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="H23" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B25" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="C25" s="9" t="str">
+        <f>'Problema 1 (enunciado)'!C8</f>
+        <v>-</v>
+      </c>
+      <c r="D25" s="24">
+        <f>'Problema 1 (enunciado)'!D8*'Problema 1 (graficos)'!G5</f>
+        <v>80</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F25" s="28">
+        <f>D25</f>
+        <v>80</v>
+      </c>
+      <c r="G25" s="22"/>
+      <c r="H25" s="28">
+        <f>D25</f>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B26" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26" s="25">
+        <f>'Problema 1 (enunciado)'!C9</f>
+        <v>80000</v>
+      </c>
+      <c r="D26" s="24">
+        <f>'Problema 1 (enunciado)'!D9*'Problema 1 (graficos)'!G6</f>
+        <v>30</v>
+      </c>
+      <c r="E26" s="22">
+        <f>C26*1.2</f>
+        <v>96000</v>
+      </c>
+      <c r="F26" s="28">
+        <f t="shared" ref="F26:F29" si="0">D26</f>
+        <v>30</v>
+      </c>
+      <c r="G26" s="25">
+        <f>C26*1.5</f>
+        <v>120000</v>
+      </c>
+      <c r="H26" s="28">
+        <f t="shared" ref="H26:H29" si="1">D26</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B27" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" s="25">
+        <f>'Problema 1 (enunciado)'!C10</f>
+        <v>20000</v>
+      </c>
+      <c r="D27" s="24">
+        <f>'Problema 1 (enunciado)'!D10*'Problema 1 (graficos)'!G7</f>
+        <v>90</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F27" s="28">
+        <f t="shared" si="0"/>
+        <v>90</v>
+      </c>
+      <c r="G27" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="H27" s="28">
+        <f t="shared" si="1"/>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B28" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C28" s="25">
+        <f>'Problema 1 (enunciado)'!C11</f>
+        <v>32000</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F28" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G28" s="25">
+        <f>'Problema 1 (enunciado)'!C26</f>
+        <v>24000</v>
+      </c>
+      <c r="H28" s="28" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B29" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="C29" s="25">
+        <f>'Problema 1 (enunciado)'!C12</f>
+        <v>60000</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F29" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v>-</v>
+      </c>
+      <c r="G29" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="H29" s="28" t="str">
+        <f t="shared" si="1"/>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B31" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C31" s="10">
+        <f>SUM(C25:C29)</f>
+        <v>192000</v>
+      </c>
+      <c r="D31" s="10">
+        <f t="shared" ref="D31:H31" si="2">SUM(D25:D29)</f>
+        <v>200</v>
+      </c>
+      <c r="E31" s="10">
+        <f t="shared" si="2"/>
+        <v>96000</v>
+      </c>
+      <c r="F31" s="10">
+        <f t="shared" si="2"/>
+        <v>200</v>
+      </c>
+      <c r="G31" s="10">
+        <f t="shared" si="2"/>
+        <v>144000</v>
+      </c>
+      <c r="H31" s="10">
+        <f t="shared" si="2"/>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="I32" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="L32" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="33" spans="2:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="B33" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="C33" s="30">
+        <f>C12*D31+C31</f>
+        <v>672000</v>
+      </c>
+      <c r="D33" s="30"/>
+      <c r="E33" s="30">
+        <f>(4000-C12)*F31+E31</f>
+        <v>416000</v>
+      </c>
+      <c r="G33" s="30"/>
+      <c r="I33" s="30">
+        <f>C33+E33+G33</f>
+        <v>1088000</v>
+      </c>
+      <c r="J33" s="30">
+        <f>I33/4000</f>
+        <v>272</v>
+      </c>
+      <c r="K33" s="30">
+        <f>I33+'Problema 1 (enunciado)'!C27</f>
+        <v>1360000</v>
+      </c>
+      <c r="L33" s="30">
+        <f>K33/4000</f>
+        <v>340</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
+        <v>54</v>
+      </c>
+      <c r="C34" s="30">
+        <f>C33/C12</f>
+        <v>280</v>
+      </c>
+      <c r="E34" s="30">
+        <f>E33/(4000-C12)</f>
+        <v>260</v>
+      </c>
+      <c r="G34" s="30"/>
+    </row>
+    <row r="36" spans="2:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="B36" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="C36" s="30">
+        <f>C12*D31+C31</f>
+        <v>672000</v>
+      </c>
+      <c r="E36" s="30">
+        <f>C12*F31+E31</f>
+        <v>576000</v>
+      </c>
+      <c r="G36" s="30">
+        <f>(6000-C12-C12)*H31+G31</f>
+        <v>384000</v>
+      </c>
+      <c r="I36" s="30">
+        <f>C36+E36+G36</f>
+        <v>1632000</v>
+      </c>
+      <c r="J36" s="30">
+        <f>I36/6000</f>
+        <v>272</v>
+      </c>
+      <c r="K36" s="30">
+        <f>I36+'Problema 1 (enunciado)'!C27+'Problema 1 (enunciado)'!C28</f>
+        <v>1980000</v>
+      </c>
+      <c r="L36" s="30">
+        <f>K36/6000</f>
+        <v>330</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B37" t="s">
+        <v>54</v>
+      </c>
+      <c r="C37" s="30">
+        <f>C36/C12</f>
+        <v>280</v>
+      </c>
+      <c r="E37" s="30">
+        <f>E36/C12</f>
+        <v>240</v>
+      </c>
+      <c r="G37" s="30">
+        <f>G36/(6000-C12-C12)</f>
+        <v>320</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="K33 K36" formula="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
A2 - Problema 2
</commit_message>
<xml_diff>
--- a/2024_1_SPCE_Avaliacao_A2_-_Felipe_Luiza_Marcius.xlsx
+++ b/2024_1_SPCE_Avaliacao_A2_-_Felipe_Luiza_Marcius.xlsx
@@ -5,18 +5,21 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mithra\Documents\FelipeFreitas\Sistemas_de_Planejamento_e_Custos_para_Engenharia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming\EngenhariaSoftwarePUCRS\Sistemas_de_Planejamento_e_Custos_para_Engenharia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A9ED4FC-6B19-4F49-AA75-99A324DBD05A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC120500-895E-45F6-835B-5DC6EF3A0282}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="16200" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Integrantes" sheetId="1" r:id="rId1"/>
     <sheet name="Problema 1 (enunciado)" sheetId="10" r:id="rId2"/>
     <sheet name="Problema 1 (calculos)" sheetId="11" r:id="rId3"/>
     <sheet name="Problema 1 (graficos)" sheetId="12" r:id="rId4"/>
+    <sheet name="Problema 2 (enunciado)" sheetId="13" r:id="rId5"/>
+    <sheet name="Problema 2 (calculos)" sheetId="14" r:id="rId6"/>
+    <sheet name="Problema 2 (graficos)" sheetId="15" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="108">
   <si>
     <t>Integrantes</t>
   </si>
@@ -222,6 +225,147 @@
   </si>
   <si>
     <t>Custo Total</t>
+  </si>
+  <si>
+    <t>Quantidade Produzida (Q)</t>
+  </si>
+  <si>
+    <t>Janeiro</t>
+  </si>
+  <si>
+    <t>Fevereiro</t>
+  </si>
+  <si>
+    <t>(peças por mês)</t>
+  </si>
+  <si>
+    <t>Custo Direto de Produção (C)</t>
+  </si>
+  <si>
+    <t>Materiais de produção</t>
+  </si>
+  <si>
+    <t>Energia Elétrica</t>
+  </si>
+  <si>
+    <t>Capacidade instalada de produção =</t>
+  </si>
+  <si>
+    <t>peças por mês por turno</t>
+  </si>
+  <si>
+    <t>Custos fixos indiretos =</t>
+  </si>
+  <si>
+    <t>em um turno</t>
+  </si>
+  <si>
+    <t>Custos fixos indiretos aditados =</t>
+  </si>
+  <si>
+    <t>para eventual turno adicional</t>
+  </si>
+  <si>
+    <t>Acrescimo preço mão de obra 2º turno =</t>
+  </si>
+  <si>
+    <t>Acrescimo preço armazenamento 2º turno março =</t>
+  </si>
+  <si>
+    <t>Objetivo de produção em Março =</t>
+  </si>
+  <si>
+    <t>peças</t>
+  </si>
+  <si>
+    <t>Custos no Mês de Março</t>
+  </si>
+  <si>
+    <t>Primeiro Turno</t>
+  </si>
+  <si>
+    <t>Segundo Turno</t>
+  </si>
+  <si>
+    <t>Indiretos</t>
+  </si>
+  <si>
+    <t>Quantidade Produzida</t>
+  </si>
+  <si>
+    <t>(A)</t>
+  </si>
+  <si>
+    <t>(D)</t>
+  </si>
+  <si>
+    <t>(I)</t>
+  </si>
+  <si>
+    <t>(E)</t>
+  </si>
+  <si>
+    <t>Diferença Qtd Unidades Jan Fev</t>
+  </si>
+  <si>
+    <t>CDU(E) =</t>
+  </si>
+  <si>
+    <t>CDU(A) =</t>
+  </si>
+  <si>
+    <t>CDU(D) =</t>
+  </si>
+  <si>
+    <t>CDU(Mo) =</t>
+  </si>
+  <si>
+    <t>CDU(Ma) =</t>
+  </si>
+  <si>
+    <t>(Ma)</t>
+  </si>
+  <si>
+    <t>(Mo)</t>
+  </si>
+  <si>
+    <t>CDU(I) =</t>
+  </si>
+  <si>
+    <t>Custo Fixo Direto ($ por mês)</t>
+  </si>
+  <si>
+    <t>Custo Variável Unitário ($ por peça)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acrescimo preço energia 2º turno = </t>
+  </si>
+  <si>
+    <t>Gráfico 1: Como os custos são fixos, podemos ver uma linearidade no gráfico; quanto mais produzimos, maior o custo direto total</t>
+  </si>
+  <si>
+    <t>Gráfico 2: Por outro lado, quanto mais unidades produzimos, a tendência (linha pontilhada) é que o preço por unidade diminua logaritmicamente, até um ponto em que a diminuição se torna imperceptível. É interessante observar uma não-linearidade no gráfico na reta após a produção de 5000 unidades, visto que este é o limite por turno e, quando há a necessidade de um 2º turno, os custos sobem minimamente até se equilibrarem novamente.</t>
+  </si>
+  <si>
+    <t>Gráficos 3-7: Não há gráficos para os custos de Ma, E, A, D ou Mo (ver legenda na página de cálculos), visto que todos são lineares e representam uma tendência similar de crescimento, embora com taxas diferentes. Custos como materiais e energia possuem custo fixo (inicial) menor, mas um crescimento maior conforme a produção aumenta. Custos como armazenagem e depreciação por outro lado são maiores inicialmente (custos fixos) mas não crescem tão rapidamente junto da produção.</t>
+  </si>
+  <si>
+    <t>Custo Direto Total Estimado =</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Custo Total Estimado = </t>
+  </si>
+  <si>
+    <t>Custo Total Unitário Estimado =</t>
+  </si>
+  <si>
+    <t>Custo Direto Total Real =</t>
+  </si>
+  <si>
+    <t>Custo Total Real =</t>
+  </si>
+  <si>
+    <t>Custo Total Unitário Real =</t>
   </si>
 </sst>
 </file>
@@ -256,15 +400,21 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -393,12 +543,33 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -468,10 +639,71 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Moeda" xfId="1" builtinId="4"/>
+  <cellStyles count="3">
+    <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -490,6 +722,2337 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Gráfico</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> 1</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Problema 2 (graficos)'!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Custo Direto Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Problema 2 (graficos)'!$A$2:$A$22</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1500</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2500</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3000</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3500</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4000</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4500</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5000</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5500</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>6000</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>6500</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>7000</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>7500</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>8000</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>8500</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>9000</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>9500</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>10000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Problema 2 (graficos)'!$B$2:$B$22</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>138000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>170500</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>203000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>235500</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>268000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>300500</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>333000</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>365500</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>398000</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>430500</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>463000</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>495500</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>528000</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>560500</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>593000</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>625500</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>658000</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>690500</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>723000</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>755500</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>788000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-9B1F-493A-8255-4D311B527BFF}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="996277343"/>
+        <c:axId val="996272063"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="996277343"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="10000"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Quantidade Produzida</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="996272063"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="996272063"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="800000"/>
+          <c:min val="100000"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Custo Direto</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> Total</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="996277343"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Gráfico</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> 2</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Problema 2 (graficos)'!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Custo Total Unitário</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="exp"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Problema 2 (graficos)'!$A$2:$A$22</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1500</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2500</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3000</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3500</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4000</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4500</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5000</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5500</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>6000</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>6500</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>7000</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>7500</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>8000</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>8500</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>9000</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>9500</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>10000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Problema 2 (graficos)'!$C$2:$C$22</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>218000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>501</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>283</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>210.33333333333334</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>174</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>152.19999999999999</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>137.66666666666666</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>127.28571428571429</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>119.5</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>113.44444444444444</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>108.6</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>113.72727272727273</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>109.66666666666667</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>106.23076923076923</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>103.28571428571429</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>100.73333333333333</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>98.5</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>96.529411764705884</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>94.777777777777771</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>93.21052631578948</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>91.8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-66C9-4CFB-A927-1B738F1F8CB8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="963554655"/>
+        <c:axId val="963545055"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="963554655"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="10000"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Quantidade Produzida</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="963545055"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="963545055"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1000"/>
+          <c:min val="-"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Custo Total Unitário</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="963554655"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>173553</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>695325</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{390FF248-877E-46AA-B5DA-15342E088612}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>23812</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>6543675</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="8" name="Chart 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5F1E70E1-11B5-E81C-C301-A34712FF6CCE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2546,4 +5109,964 @@
     <ignoredError sqref="K33 K36" formula="1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7218494D-15F9-4F44-9285-D2AB202B24F1}">
+  <dimension ref="B2:D27"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="34.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="28" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B2" s="34" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" ht="3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C4" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" s="38" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" ht="3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C6" s="39">
+        <v>3000</v>
+      </c>
+      <c r="D6" s="39">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" ht="3" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B8" s="36" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D8" s="36" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" ht="3" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C10" s="38" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="35" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" ht="3" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B12" s="32" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" s="31">
+        <v>60000</v>
+      </c>
+      <c r="D12" s="33">
+        <v>80000</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B13" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="C13" s="31">
+        <v>85000</v>
+      </c>
+      <c r="D13" s="33">
+        <v>110000</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B14" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="31">
+        <v>46000</v>
+      </c>
+      <c r="D14" s="33">
+        <v>53000</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B15" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="31">
+        <v>68000</v>
+      </c>
+      <c r="D15" s="33">
+        <v>73000</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B16" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="31">
+        <v>74000</v>
+      </c>
+      <c r="D16" s="33">
+        <v>82000</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="43"/>
+      <c r="C17" s="44"/>
+      <c r="D17" s="44"/>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B18" s="46" t="s">
+        <v>48</v>
+      </c>
+      <c r="C18" s="12">
+        <f>SUM(C12:C16)</f>
+        <v>333000</v>
+      </c>
+      <c r="D18" s="12">
+        <f>SUM(D12:D16)</f>
+        <v>398000</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B19" s="46"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B20" s="45" t="s">
+        <v>87</v>
+      </c>
+      <c r="C20" s="12">
+        <f>D6-C6</f>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" s="40">
+        <v>5000</v>
+      </c>
+      <c r="D21" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>70</v>
+      </c>
+      <c r="C22" s="40">
+        <v>80000</v>
+      </c>
+      <c r="D22" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>72</v>
+      </c>
+      <c r="C23" s="40">
+        <v>50000</v>
+      </c>
+      <c r="D23" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>74</v>
+      </c>
+      <c r="C24" s="41">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>98</v>
+      </c>
+      <c r="C25" s="41">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>75</v>
+      </c>
+      <c r="D26" s="12">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>76</v>
+      </c>
+      <c r="C27" s="40">
+        <v>8000</v>
+      </c>
+      <c r="D27" t="s">
+        <v>77</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72E9EE7-BF61-4C58-900F-78527D3312AC}">
+  <dimension ref="A2:G30"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="23.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B2" s="36" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="3" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C4" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E4" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="F4" s="36" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C5" s="37"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C6" s="38" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="E6" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="35" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="3" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B8" s="32" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" s="54">
+        <f>C24</f>
+        <v>0</v>
+      </c>
+      <c r="D8" s="39">
+        <f>D24</f>
+        <v>20</v>
+      </c>
+      <c r="E8" s="54" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="39">
+        <f>D8</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>86</v>
+      </c>
+      <c r="B9" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="C9" s="54">
+        <f>C25</f>
+        <v>10000</v>
+      </c>
+      <c r="D9" s="39">
+        <f>D25</f>
+        <v>25</v>
+      </c>
+      <c r="E9" s="54" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="39">
+        <f>D9*(1+'Problema 2 (enunciado)'!C25)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B10" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="54">
+        <f>C26</f>
+        <v>25000</v>
+      </c>
+      <c r="D10" s="39">
+        <f>D26</f>
+        <v>7</v>
+      </c>
+      <c r="E10" s="54">
+        <f>'Problema 2 (enunciado)'!D26</f>
+        <v>5000</v>
+      </c>
+      <c r="F10" s="39">
+        <f>D10</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B11" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="54">
+        <f>C27</f>
+        <v>53000</v>
+      </c>
+      <c r="D11" s="39">
+        <f>D27</f>
+        <v>5</v>
+      </c>
+      <c r="E11" s="54" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="39">
+        <f>D11</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>94</v>
+      </c>
+      <c r="B12" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="54">
+        <f>C28</f>
+        <v>50000</v>
+      </c>
+      <c r="D12" s="39">
+        <f>D28</f>
+        <v>8</v>
+      </c>
+      <c r="E12" s="54">
+        <f>C12*(1+'Problema 2 (enunciado)'!C24)</f>
+        <v>75000</v>
+      </c>
+      <c r="F12" s="39">
+        <f>D12*(1+'Problema 2 (enunciado)'!C24)</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B13" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="C13" s="54">
+        <f>C29</f>
+        <v>80000</v>
+      </c>
+      <c r="D13" s="39">
+        <f>D29</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="54">
+        <f>'Problema 2 (enunciado)'!C23</f>
+        <v>50000</v>
+      </c>
+      <c r="F13" s="39" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C14" s="40"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="43"/>
+      <c r="B15" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="42">
+        <f>SUM(C8:C13)</f>
+        <v>218000</v>
+      </c>
+      <c r="D15" s="55">
+        <f>SUM(D8:D13)</f>
+        <v>65</v>
+      </c>
+      <c r="E15" s="55">
+        <f>SUM(E8:E13)</f>
+        <v>130000</v>
+      </c>
+      <c r="F15" s="56">
+        <f>SUM(F8:F13)</f>
+        <v>74</v>
+      </c>
+      <c r="G15" s="43"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C16" s="40"/>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B17" t="str">
+        <f>"Q1 = "&amp;'Problema 2 (enunciado)'!C6 &amp; "| C1 = " &amp; 'Problema 2 (enunciado)'!C18</f>
+        <v>Q1 = 3000| C1 = 333000</v>
+      </c>
+      <c r="C17" s="41" t="str">
+        <f>"Eq1 - Eq2 -&gt; " &amp; 'Problema 2 (enunciado)'!D18-'Problema 2 (enunciado)'!C18&amp;" = " &amp; 'Problema 2 (enunciado)'!D6-'Problema 2 (enunciado)'!C6 &amp; " x V1 -&gt; V1 = "</f>
+        <v xml:space="preserve">Eq1 - Eq2 -&gt; 65000 = 1000 x V1 -&gt; V1 = </v>
+      </c>
+      <c r="D17" s="47">
+        <f>('Problema 2 (enunciado)'!D18-'Problema 2 (enunciado)'!C18)/('Problema 2 (enunciado)'!D6-'Problema 2 (enunciado)'!C6)</f>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B18" t="str">
+        <f>"Q1 = "&amp;'Problema 2 (enunciado)'!D6 &amp; "| C1 = " &amp; 'Problema 2 (enunciado)'!D18</f>
+        <v>Q1 = 4000| C1 = 398000</v>
+      </c>
+      <c r="C18" s="41" t="str">
+        <f>"F1 = " &amp; 'Problema 2 (enunciado)'!C18 &amp; " - " &amp; 'Problema 2 (enunciado)'!C6 &amp; " * " &amp; 'Problema 2 (calculos)'!D17 &amp; " = "</f>
+        <v xml:space="preserve">F1 = 333000 - 3000 * 65 = </v>
+      </c>
+      <c r="D18" s="48">
+        <f>'Problema 2 (enunciado)'!C18-'Problema 2 (enunciado)'!C6*'Problema 2 (calculos)'!D17</f>
+        <v>138000</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>102</v>
+      </c>
+      <c r="C19" s="40">
+        <f>'Problema 2 (graficos)'!B18</f>
+        <v>658000</v>
+      </c>
+      <c r="D19" t="s">
+        <v>105</v>
+      </c>
+      <c r="E19" s="12">
+        <f>C15+E15</f>
+        <v>348000</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>103</v>
+      </c>
+      <c r="C20" s="12">
+        <f>'Problema 2 (graficos)'!B18+'Problema 2 (enunciado)'!C22+'Problema 2 (enunciado)'!C23</f>
+        <v>788000</v>
+      </c>
+      <c r="D20" t="s">
+        <v>106</v>
+      </c>
+      <c r="E20" s="12">
+        <f>E19-C13-E13</f>
+        <v>218000</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>104</v>
+      </c>
+      <c r="C21">
+        <f>C20/'Problema 2 (enunciado)'!C27</f>
+        <v>98.5</v>
+      </c>
+      <c r="D21" t="s">
+        <v>107</v>
+      </c>
+      <c r="E21">
+        <f>((C15+D15*5000)+(E15+F15*3000))/8000</f>
+        <v>111.875</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C23" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B24" s="53" t="s">
+        <v>92</v>
+      </c>
+      <c r="C24" s="12">
+        <f>'Problema 2 (enunciado)'!C12-'Problema 2 (enunciado)'!$C$6*D24</f>
+        <v>0</v>
+      </c>
+      <c r="D24" s="12">
+        <f>('Problema 2 (enunciado)'!D12-'Problema 2 (enunciado)'!C12)/'Problema 2 (enunciado)'!$C$20</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="53" t="s">
+        <v>88</v>
+      </c>
+      <c r="C25" s="12">
+        <f>'Problema 2 (enunciado)'!C13-'Problema 2 (enunciado)'!$C$6*D25</f>
+        <v>10000</v>
+      </c>
+      <c r="D25" s="12">
+        <f>('Problema 2 (enunciado)'!D13-'Problema 2 (enunciado)'!C13)/'Problema 2 (enunciado)'!$C$20</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B26" s="53" t="s">
+        <v>89</v>
+      </c>
+      <c r="C26" s="12">
+        <f>'Problema 2 (enunciado)'!C14-'Problema 2 (enunciado)'!$C$6*D26</f>
+        <v>25000</v>
+      </c>
+      <c r="D26" s="12">
+        <f>('Problema 2 (enunciado)'!D14-'Problema 2 (enunciado)'!C14)/'Problema 2 (enunciado)'!$C$20</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B27" s="53" t="s">
+        <v>90</v>
+      </c>
+      <c r="C27" s="12">
+        <f>'Problema 2 (enunciado)'!C15-'Problema 2 (enunciado)'!$C$6*D27</f>
+        <v>53000</v>
+      </c>
+      <c r="D27" s="12">
+        <f>('Problema 2 (enunciado)'!D15-'Problema 2 (enunciado)'!C15)/'Problema 2 (enunciado)'!$C$20</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B28" s="53" t="s">
+        <v>91</v>
+      </c>
+      <c r="C28" s="12">
+        <f>'Problema 2 (enunciado)'!C16-'Problema 2 (enunciado)'!$C$6*D28</f>
+        <v>50000</v>
+      </c>
+      <c r="D28" s="12">
+        <f>('Problema 2 (enunciado)'!D16-'Problema 2 (enunciado)'!C16)/'Problema 2 (enunciado)'!$C$20</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B29" s="53" t="s">
+        <v>95</v>
+      </c>
+      <c r="C29" s="12">
+        <f>'Problema 2 (enunciado)'!C22</f>
+        <v>80000</v>
+      </c>
+      <c r="D29" s="12">
+        <f>('Problema 2 (enunciado)'!D17-'Problema 2 (enunciado)'!C17)/'Problema 2 (enunciado)'!$C$20</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B30" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C30" s="12">
+        <f>SUM(C24:C29)</f>
+        <v>218000</v>
+      </c>
+      <c r="D30" s="12">
+        <f>SUM(D24:D29)</f>
+        <v>65</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="F9" formula="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B864A96-F0B9-4EB4-8927-6C28AF2B9792}">
+  <dimension ref="A1:E28"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.5703125" customWidth="1"/>
+    <col min="5" max="5" width="98.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A2</f>
+        <v>138000</v>
+      </c>
+      <c r="C2" s="12">
+        <f>(B2+'Problema 2 (enunciado)'!$C$22)*1</f>
+        <v>218000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>500</v>
+      </c>
+      <c r="B3">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A3</f>
+        <v>170500</v>
+      </c>
+      <c r="C3" s="12">
+        <f>(B3+'Problema 2 (enunciado)'!$C$22)/A3</f>
+        <v>501</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>1000</v>
+      </c>
+      <c r="B4">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A4</f>
+        <v>203000</v>
+      </c>
+      <c r="C4" s="12">
+        <f>(B4+'Problema 2 (enunciado)'!$C$22)/A4</f>
+        <v>283</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>1500</v>
+      </c>
+      <c r="B5">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A5</f>
+        <v>235500</v>
+      </c>
+      <c r="C5" s="12">
+        <f>(B5+'Problema 2 (enunciado)'!$C$22)/A5</f>
+        <v>210.33333333333334</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2000</v>
+      </c>
+      <c r="B6">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A6</f>
+        <v>268000</v>
+      </c>
+      <c r="C6" s="12">
+        <f>(B6+'Problema 2 (enunciado)'!$C$22)/A6</f>
+        <v>174</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2500</v>
+      </c>
+      <c r="B7">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A7</f>
+        <v>300500</v>
+      </c>
+      <c r="C7" s="12">
+        <f>(B7+'Problema 2 (enunciado)'!$C$22)/A7</f>
+        <v>152.19999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>3000</v>
+      </c>
+      <c r="B8">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A8</f>
+        <v>333000</v>
+      </c>
+      <c r="C8" s="12">
+        <f>(B8+'Problema 2 (enunciado)'!$C$22)/A8</f>
+        <v>137.66666666666666</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>3500</v>
+      </c>
+      <c r="B9">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A9</f>
+        <v>365500</v>
+      </c>
+      <c r="C9" s="12">
+        <f>(B9+'Problema 2 (enunciado)'!$C$22)/A9</f>
+        <v>127.28571428571429</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>4000</v>
+      </c>
+      <c r="B10">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A10</f>
+        <v>398000</v>
+      </c>
+      <c r="C10" s="12">
+        <f>(B10+'Problema 2 (enunciado)'!$C$22)/A10</f>
+        <v>119.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>4500</v>
+      </c>
+      <c r="B11">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A11</f>
+        <v>430500</v>
+      </c>
+      <c r="C11" s="12">
+        <f>(B11+'Problema 2 (enunciado)'!$C$22)/A11</f>
+        <v>113.44444444444444</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="50">
+        <v>5000</v>
+      </c>
+      <c r="B12" s="50">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A12</f>
+        <v>463000</v>
+      </c>
+      <c r="C12" s="51">
+        <f>(B12+'Problema 2 (enunciado)'!$C$22)/A12</f>
+        <v>108.6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>5500</v>
+      </c>
+      <c r="B13">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A13</f>
+        <v>495500</v>
+      </c>
+      <c r="C13" s="12">
+        <f>(B13+'Problema 2 (enunciado)'!$C$22+'Problema 2 (enunciado)'!$C$23)/'Problema 2 (graficos)'!A13</f>
+        <v>113.72727272727273</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>6000</v>
+      </c>
+      <c r="B14">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A14</f>
+        <v>528000</v>
+      </c>
+      <c r="C14" s="12">
+        <f>(B14+'Problema 2 (enunciado)'!$C$22+'Problema 2 (enunciado)'!$C$23)/'Problema 2 (graficos)'!A14</f>
+        <v>109.66666666666667</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>6500</v>
+      </c>
+      <c r="B15">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A15</f>
+        <v>560500</v>
+      </c>
+      <c r="C15" s="12">
+        <f>(B15+'Problema 2 (enunciado)'!$C$22+'Problema 2 (enunciado)'!$C$23)/'Problema 2 (graficos)'!A15</f>
+        <v>106.23076923076923</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>7000</v>
+      </c>
+      <c r="B16">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A16</f>
+        <v>593000</v>
+      </c>
+      <c r="C16" s="12">
+        <f>(B16+'Problema 2 (enunciado)'!$C$22+'Problema 2 (enunciado)'!$C$23)/'Problema 2 (graficos)'!A16</f>
+        <v>103.28571428571429</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>7500</v>
+      </c>
+      <c r="B17">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A17</f>
+        <v>625500</v>
+      </c>
+      <c r="C17" s="12">
+        <f>(B17+'Problema 2 (enunciado)'!$C$22+'Problema 2 (enunciado)'!$C$23)/'Problema 2 (graficos)'!A17</f>
+        <v>100.73333333333333</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>8000</v>
+      </c>
+      <c r="B18" s="49">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A18</f>
+        <v>658000</v>
+      </c>
+      <c r="C18" s="52">
+        <f>(B18+'Problema 2 (enunciado)'!$C$22+'Problema 2 (enunciado)'!$C$23)/'Problema 2 (graficos)'!A18</f>
+        <v>98.5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>8500</v>
+      </c>
+      <c r="B19">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A19</f>
+        <v>690500</v>
+      </c>
+      <c r="C19" s="12">
+        <f>(B19+'Problema 2 (enunciado)'!$C$22+'Problema 2 (enunciado)'!$C$23)/'Problema 2 (graficos)'!A19</f>
+        <v>96.529411764705884</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>9000</v>
+      </c>
+      <c r="B20">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A20</f>
+        <v>723000</v>
+      </c>
+      <c r="C20" s="12">
+        <f>(B20+'Problema 2 (enunciado)'!$C$22+'Problema 2 (enunciado)'!$C$23)/'Problema 2 (graficos)'!A20</f>
+        <v>94.777777777777771</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>9500</v>
+      </c>
+      <c r="B21">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A21</f>
+        <v>755500</v>
+      </c>
+      <c r="C21" s="12">
+        <f>(B21+'Problema 2 (enunciado)'!$C$22+'Problema 2 (enunciado)'!$C$23)/'Problema 2 (graficos)'!A21</f>
+        <v>93.21052631578948</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>10000</v>
+      </c>
+      <c r="B22">
+        <f>'Problema 2 (calculos)'!$D$18+'Problema 2 (calculos)'!$D$17*'Problema 2 (graficos)'!A22</f>
+        <v>788000</v>
+      </c>
+      <c r="C22" s="12">
+        <f>(B22+'Problema 2 (enunciado)'!$C$22+'Problema 2 (enunciado)'!$C$23)/'Problema 2 (graficos)'!A22</f>
+        <v>91.8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="E24" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="E26" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="E28" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>